<commit_message>
Render absences as "відсутній" in bot messages
</commit_message>
<xml_diff>
--- a/examples/Безпека інформаційних систем - Чопоров С.В..xlsx
+++ b/examples/Безпека інформаційних систем - Чопоров С.В..xlsx
@@ -1,13 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schop\Documents\eu_grades\examples\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7A9EB1-9EA5-42D3-AA2F-B9744C810DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="222" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="223" sheetId="2" r:id="rId6"/>
+    <sheet name="222" sheetId="1" r:id="rId1"/>
+    <sheet name="223" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -149,38 +158,43 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd.MM.yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="6">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF444746"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
@@ -190,50 +204,44 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -241,7 +249,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -431,22 +439,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="2.75"/>
-    <col customWidth="1" min="2" max="2" width="30.0"/>
-    <col customWidth="1" min="3" max="3" width="21.13"/>
+    <col min="1" max="1" width="2.77734375" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,28 +468,28 @@
         <v>2</v>
       </c>
       <c r="D1" s="2">
-        <v>46154.0</v>
+        <v>46153</v>
       </c>
       <c r="E1" s="2">
-        <v>46154.0</v>
+        <v>46154</v>
       </c>
       <c r="F1" s="2">
-        <v>46155.0</v>
+        <v>46155</v>
       </c>
       <c r="G1" s="2">
-        <v>46156.0</v>
+        <v>46156</v>
       </c>
       <c r="H1" s="2">
-        <v>46157.0</v>
+        <v>46157</v>
       </c>
       <c r="I1" s="2">
-        <v>46158.0</v>
+        <v>46158</v>
       </c>
       <c r="J1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10">
       <c r="A2" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -496,16 +507,16 @@
         <v>5</v>
       </c>
       <c r="G2" s="6">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H2" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="I2" s="7"/>
-    </row>
-    <row r="3">
+        <v>2</v>
+      </c>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>6</v>
@@ -514,21 +525,21 @@
         <v>7</v>
       </c>
       <c r="D3" s="6">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="E3" s="6">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="F3" s="6">
-        <v>11.0</v>
-      </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-    </row>
-    <row r="4">
+        <v>11</v>
+      </c>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="4">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>8</v>
@@ -537,19 +548,19 @@
         <v>9</v>
       </c>
       <c r="D4" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="E4" s="7"/>
+        <v>4</v>
+      </c>
+      <c r="E4" s="6"/>
       <c r="F4" s="6">
-        <v>6.0</v>
-      </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5">
+        <v>6</v>
+      </c>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" s="4">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>10</v>
@@ -557,16 +568,16 @@
       <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-    </row>
-    <row r="6">
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="4">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>12</v>
@@ -580,14 +591,14 @@
       <c r="E6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-    </row>
-    <row r="7">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="4">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>14</v>
@@ -595,16 +606,16 @@
       <c r="C7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8">
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" s="4">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>16</v>
@@ -613,21 +624,21 @@
         <v>17</v>
       </c>
       <c r="D8" s="6">
-        <v>7.0</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>7</v>
+      </c>
+      <c r="E8" s="6"/>
       <c r="F8" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="G8" s="7"/>
+        <v>9</v>
+      </c>
+      <c r="G8" s="6"/>
       <c r="H8" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="I8" s="7"/>
-    </row>
-    <row r="9">
+        <v>9</v>
+      </c>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" s="4">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>18</v>
@@ -635,16 +646,16 @@
       <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-    </row>
-    <row r="10">
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" s="4">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>20</v>
@@ -652,16 +663,16 @@
       <c r="C10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11">
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>22</v>
@@ -670,41 +681,42 @@
         <v>23</v>
       </c>
       <c r="D11" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="E11" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="E11" s="6"/>
       <c r="F11" s="6">
-        <v>12.0</v>
-      </c>
-      <c r="G11" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="G11" s="6"/>
       <c r="H11" s="6">
-        <v>12.0</v>
-      </c>
-      <c r="I11" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="I11" s="6"/>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:I11">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:I11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"в,1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="2.88"/>
-    <col customWidth="1" min="2" max="2" width="30.38"/>
-    <col customWidth="1" min="3" max="3" width="20.63"/>
+    <col min="1" max="1" width="2.88671875" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -715,27 +727,27 @@
         <v>2</v>
       </c>
       <c r="D1" s="2">
-        <v>46154.0</v>
+        <v>46153</v>
       </c>
       <c r="E1" s="2">
-        <v>46154.0</v>
+        <v>46154</v>
       </c>
       <c r="F1" s="2">
-        <v>46155.0</v>
+        <v>46155</v>
       </c>
       <c r="G1" s="2">
-        <v>46156.0</v>
+        <v>46156</v>
       </c>
       <c r="H1" s="2">
-        <v>46157.0</v>
+        <v>46157</v>
       </c>
       <c r="I1" s="2">
-        <v>46158.0</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>46158</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>24</v>
@@ -744,23 +756,23 @@
         <v>25</v>
       </c>
       <c r="D2" s="6">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E2" s="6">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F2" s="6">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-    </row>
-    <row r="3">
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>26</v>
@@ -768,16 +780,16 @@
       <c r="C3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-    </row>
-    <row r="4">
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="4">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>28</v>
@@ -785,18 +797,18 @@
       <c r="C4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
       <c r="G4" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5">
+        <v>2</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="4">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>30</v>
@@ -804,18 +816,18 @@
       <c r="C5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
       <c r="H5" s="6">
-        <v>12.0</v>
-      </c>
-      <c r="I5" s="7"/>
-    </row>
-    <row r="6">
+        <v>12</v>
+      </c>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" s="4">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>32</v>
@@ -823,18 +835,18 @@
       <c r="C6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="7"/>
+      <c r="D6" s="6"/>
       <c r="E6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-    </row>
-    <row r="7">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" s="4">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>34</v>
@@ -842,18 +854,18 @@
       <c r="C7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
       <c r="G7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8">
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" s="4">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>36</v>
@@ -862,19 +874,19 @@
         <v>37</v>
       </c>
       <c r="D8" s="6">
-        <v>10.0</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="E8" s="6"/>
       <c r="F8" s="6">
-        <v>12.0</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-    </row>
-    <row r="9">
+        <v>12</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="4">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>38</v>
@@ -882,18 +894,18 @@
       <c r="C9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
       <c r="H9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="7"/>
-    </row>
-    <row r="10">
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" s="4">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>40</v>
@@ -901,16 +913,16 @@
       <c r="C10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11">
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>42</v>
@@ -919,24 +931,24 @@
         <v>43</v>
       </c>
       <c r="D11" s="6">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="E11" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="6">
-        <v>10.0</v>
-      </c>
-      <c r="I11" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="I11" s="6"/>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:I11">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:I11" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"в,1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>